<commit_message>
test(load): run Load tests
</commit_message>
<xml_diff>
--- a/testing/load-tests/Load_Test_Report.xlsx
+++ b/testing/load-tests/Load_Test_Report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1036" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="79">
   <si>
     <t>GROWMARK BACKEND — LOAD TEST REPORT</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Start Time</t>
   </si>
   <si>
-    <t>8/7/2026, 2:26:39 PM</t>
+    <t>8/7/2026, 2:41:01 PM</t>
   </si>
   <si>
     <t>When the test started</t>
@@ -66,7 +66,7 @@
     <t>End Time</t>
   </si>
   <si>
-    <t>8/7/2026, 2:27:40 PM</t>
+    <t>8/7/2026, 2:42:02 PM</t>
   </si>
   <si>
     <t>When the test finished</t>
@@ -84,7 +84,7 @@
     <t>Average RPS</t>
   </si>
   <si>
-    <t>545.68</t>
+    <t>1205.62</t>
   </si>
   <si>
     <t>Average requests served per second</t>
@@ -108,7 +108,7 @@
     <t>Average Response Time</t>
   </si>
   <si>
-    <t>459.19 ms</t>
+    <t>248.58 ms</t>
   </si>
   <si>
     <t>Mean time server took to respond</t>
@@ -117,7 +117,7 @@
     <t>Min Response Time</t>
   </si>
   <si>
-    <t>88 ms</t>
+    <t>58 ms</t>
   </si>
   <si>
     <t>Fastest response observed</t>
@@ -126,7 +126,7 @@
     <t>Max Response Time</t>
   </si>
   <si>
-    <t>9920 ms</t>
+    <t>9902 ms</t>
   </si>
   <si>
     <t>Slowest response observed</t>
@@ -135,7 +135,7 @@
     <t>p50 (Median)</t>
   </si>
   <si>
-    <t>279 ms</t>
+    <t>127 ms</t>
   </si>
   <si>
     <t>50% of requests responded within this time</t>
@@ -144,7 +144,7 @@
     <t>p75</t>
   </si>
   <si>
-    <t>510 ms</t>
+    <t>253 ms</t>
   </si>
   <si>
     <t>75% of requests responded within this time</t>
@@ -153,7 +153,7 @@
     <t>p99</t>
   </si>
   <si>
-    <t>3787 ms</t>
+    <t>1591 ms</t>
   </si>
   <si>
     <t>99% of requests responded within this time</t>
@@ -195,7 +195,7 @@
     <t>Total Bytes Read</t>
   </si>
   <si>
-    <t>33192.69 KB</t>
+    <t>74578.80 KB</t>
   </si>
   <si>
     <t>Total data received from the server</t>
@@ -204,7 +204,7 @@
     <t>Average Throughput</t>
   </si>
   <si>
-    <t>562.57 KB/s</t>
+    <t>1243.02 KB/s</t>
   </si>
   <si>
     <t>Average data received per second</t>
@@ -246,10 +246,10 @@
     <t>Active — Some Errors</t>
   </si>
   <si>
-    <t>107.3</t>
-  </si>
-  <si>
-    <t>459.19</t>
+    <t>241.1</t>
+  </si>
+  <si>
+    <t>248.58</t>
   </si>
 </sst>
 </file>
@@ -867,7 +867,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="6">
-        <v>32195</v>
+        <v>72337</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>21</v>
@@ -889,7 +889,7 @@
         <v>25</v>
       </c>
       <c r="B13" s="6">
-        <v>927</v>
+        <v>1675</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>26</v>
@@ -900,7 +900,7 @@
         <v>27</v>
       </c>
       <c r="B14" s="9">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>28</v>
@@ -1002,7 +1002,7 @@
         <v>52</v>
       </c>
       <c r="B24" s="6">
-        <v>324</v>
+        <v>17</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>53</v>
@@ -1013,7 +1013,7 @@
         <v>54</v>
       </c>
       <c r="B25" s="9">
-        <v>324</v>
+        <v>17</v>
       </c>
       <c r="C25" s="10" t="s">
         <v>55</v>
@@ -1024,7 +1024,7 @@
         <v>56</v>
       </c>
       <c r="B26" s="6">
-        <v>32195</v>
+        <v>72337</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>57</v>
@@ -1075,7 +1075,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1137,7 +1137,7 @@
         <v>300</v>
       </c>
       <c r="C5" s="9">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="D5" s="9">
         <v>0</v>
@@ -1154,7 +1154,7 @@
         <v>300</v>
       </c>
       <c r="C6" s="6">
-        <v>0</v>
+        <v>1199</v>
       </c>
       <c r="D6" s="6">
         <v>0</v>
@@ -1171,7 +1171,7 @@
         <v>300</v>
       </c>
       <c r="C7" s="9">
-        <v>0</v>
+        <v>1072</v>
       </c>
       <c r="D7" s="9">
         <v>0</v>
@@ -1188,7 +1188,7 @@
         <v>300</v>
       </c>
       <c r="C8" s="6">
-        <v>0</v>
+        <v>1226</v>
       </c>
       <c r="D8" s="6">
         <v>0</v>
@@ -1205,7 +1205,7 @@
         <v>300</v>
       </c>
       <c r="C9" s="9">
-        <v>0</v>
+        <v>1235</v>
       </c>
       <c r="D9" s="9">
         <v>0</v>
@@ -1222,7 +1222,7 @@
         <v>300</v>
       </c>
       <c r="C10" s="6">
-        <v>0</v>
+        <v>935</v>
       </c>
       <c r="D10" s="6">
         <v>0</v>
@@ -1239,7 +1239,7 @@
         <v>300</v>
       </c>
       <c r="C11" s="9">
-        <v>0</v>
+        <v>1179</v>
       </c>
       <c r="D11" s="9">
         <v>0</v>
@@ -1256,7 +1256,7 @@
         <v>300</v>
       </c>
       <c r="C12" s="6">
-        <v>0</v>
+        <v>1162</v>
       </c>
       <c r="D12" s="6">
         <v>0</v>
@@ -1273,7 +1273,7 @@
         <v>300</v>
       </c>
       <c r="C13" s="9">
-        <v>0</v>
+        <v>1081</v>
       </c>
       <c r="D13" s="9">
         <v>0</v>
@@ -1290,7 +1290,7 @@
         <v>300</v>
       </c>
       <c r="C14" s="6">
-        <v>0</v>
+        <v>340</v>
       </c>
       <c r="D14" s="6">
         <v>0</v>
@@ -1307,7 +1307,7 @@
         <v>300</v>
       </c>
       <c r="C15" s="9">
-        <v>0</v>
+        <v>376</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
@@ -1324,7 +1324,7 @@
         <v>300</v>
       </c>
       <c r="C16" s="6">
-        <v>436</v>
+        <v>827</v>
       </c>
       <c r="D16" s="6">
         <v>0</v>
@@ -1341,7 +1341,7 @@
         <v>300</v>
       </c>
       <c r="C17" s="9">
-        <v>432</v>
+        <v>850</v>
       </c>
       <c r="D17" s="9">
         <v>0</v>
@@ -1358,7 +1358,7 @@
         <v>300</v>
       </c>
       <c r="C18" s="6">
-        <v>99</v>
+        <v>755</v>
       </c>
       <c r="D18" s="6">
         <v>0</v>
@@ -1375,7 +1375,7 @@
         <v>300</v>
       </c>
       <c r="C19" s="9">
-        <v>230</v>
+        <v>840</v>
       </c>
       <c r="D19" s="9">
         <v>0</v>
@@ -1392,7 +1392,7 @@
         <v>300</v>
       </c>
       <c r="C20" s="6">
-        <v>252</v>
+        <v>939</v>
       </c>
       <c r="D20" s="6">
         <v>0</v>
@@ -1409,7 +1409,7 @@
         <v>300</v>
       </c>
       <c r="C21" s="9">
-        <v>605</v>
+        <v>713</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
@@ -1426,7 +1426,7 @@
         <v>300</v>
       </c>
       <c r="C22" s="6">
-        <v>718</v>
+        <v>966</v>
       </c>
       <c r="D22" s="6">
         <v>0</v>
@@ -1443,7 +1443,7 @@
         <v>300</v>
       </c>
       <c r="C23" s="9">
-        <v>806</v>
+        <v>1138</v>
       </c>
       <c r="D23" s="9">
         <v>0</v>
@@ -1460,7 +1460,7 @@
         <v>300</v>
       </c>
       <c r="C24" s="6">
-        <v>726</v>
+        <v>1128</v>
       </c>
       <c r="D24" s="6">
         <v>0</v>
@@ -1477,7 +1477,7 @@
         <v>300</v>
       </c>
       <c r="C25" s="9">
-        <v>798</v>
+        <v>1247</v>
       </c>
       <c r="D25" s="9">
         <v>0</v>
@@ -1494,7 +1494,7 @@
         <v>300</v>
       </c>
       <c r="C26" s="6">
-        <v>686</v>
+        <v>1149</v>
       </c>
       <c r="D26" s="6">
         <v>0</v>
@@ -1511,7 +1511,7 @@
         <v>300</v>
       </c>
       <c r="C27" s="9">
-        <v>789</v>
+        <v>1402</v>
       </c>
       <c r="D27" s="9">
         <v>0</v>
@@ -1528,7 +1528,7 @@
         <v>300</v>
       </c>
       <c r="C28" s="6">
-        <v>798</v>
+        <v>1367</v>
       </c>
       <c r="D28" s="6">
         <v>0</v>
@@ -1545,7 +1545,7 @@
         <v>300</v>
       </c>
       <c r="C29" s="9">
-        <v>818</v>
+        <v>1538</v>
       </c>
       <c r="D29" s="9">
         <v>0</v>
@@ -1562,7 +1562,7 @@
         <v>300</v>
       </c>
       <c r="C30" s="6">
-        <v>644</v>
+        <v>1405</v>
       </c>
       <c r="D30" s="6">
         <v>0</v>
@@ -1579,7 +1579,7 @@
         <v>300</v>
       </c>
       <c r="C31" s="9">
-        <v>508</v>
+        <v>1494</v>
       </c>
       <c r="D31" s="9">
         <v>0</v>
@@ -1596,7 +1596,7 @@
         <v>300</v>
       </c>
       <c r="C32" s="6">
-        <v>751</v>
+        <v>1558</v>
       </c>
       <c r="D32" s="6">
         <v>0</v>
@@ -1613,7 +1613,7 @@
         <v>300</v>
       </c>
       <c r="C33" s="9">
-        <v>700</v>
+        <v>1370</v>
       </c>
       <c r="D33" s="9">
         <v>0</v>
@@ -1630,7 +1630,7 @@
         <v>300</v>
       </c>
       <c r="C34" s="6">
-        <v>719</v>
+        <v>815</v>
       </c>
       <c r="D34" s="6">
         <v>0</v>
@@ -1647,7 +1647,7 @@
         <v>300</v>
       </c>
       <c r="C35" s="9">
-        <v>583</v>
+        <v>1043</v>
       </c>
       <c r="D35" s="9">
         <v>0</v>
@@ -1664,7 +1664,7 @@
         <v>300</v>
       </c>
       <c r="C36" s="6">
-        <v>272</v>
+        <v>1287</v>
       </c>
       <c r="D36" s="6">
         <v>0</v>
@@ -1681,7 +1681,7 @@
         <v>300</v>
       </c>
       <c r="C37" s="9">
-        <v>297</v>
+        <v>1322</v>
       </c>
       <c r="D37" s="9">
         <v>0</v>
@@ -1698,7 +1698,7 @@
         <v>300</v>
       </c>
       <c r="C38" s="6">
-        <v>521</v>
+        <v>1451</v>
       </c>
       <c r="D38" s="6">
         <v>0</v>
@@ -1715,7 +1715,7 @@
         <v>300</v>
       </c>
       <c r="C39" s="9">
-        <v>823</v>
+        <v>1513</v>
       </c>
       <c r="D39" s="9">
         <v>0</v>
@@ -1732,7 +1732,7 @@
         <v>300</v>
       </c>
       <c r="C40" s="6">
-        <v>798</v>
+        <v>1443</v>
       </c>
       <c r="D40" s="6">
         <v>0</v>
@@ -1749,7 +1749,7 @@
         <v>300</v>
       </c>
       <c r="C41" s="9">
-        <v>733</v>
+        <v>1215</v>
       </c>
       <c r="D41" s="9">
         <v>0</v>
@@ -1766,7 +1766,7 @@
         <v>300</v>
       </c>
       <c r="C42" s="6">
-        <v>813</v>
+        <v>1466</v>
       </c>
       <c r="D42" s="6">
         <v>0</v>
@@ -1783,7 +1783,7 @@
         <v>300</v>
       </c>
       <c r="C43" s="9">
-        <v>902</v>
+        <v>1472</v>
       </c>
       <c r="D43" s="9">
         <v>0</v>
@@ -1800,7 +1800,7 @@
         <v>300</v>
       </c>
       <c r="C44" s="6">
-        <v>621</v>
+        <v>1582</v>
       </c>
       <c r="D44" s="6">
         <v>0</v>
@@ -1817,7 +1817,7 @@
         <v>300</v>
       </c>
       <c r="C45" s="9">
-        <v>702</v>
+        <v>1565</v>
       </c>
       <c r="D45" s="9">
         <v>0</v>
@@ -1834,7 +1834,7 @@
         <v>300</v>
       </c>
       <c r="C46" s="6">
-        <v>799</v>
+        <v>1326</v>
       </c>
       <c r="D46" s="6">
         <v>0</v>
@@ -1851,7 +1851,7 @@
         <v>300</v>
       </c>
       <c r="C47" s="9">
-        <v>695</v>
+        <v>1606</v>
       </c>
       <c r="D47" s="9">
         <v>0</v>
@@ -1868,7 +1868,7 @@
         <v>300</v>
       </c>
       <c r="C48" s="6">
-        <v>802</v>
+        <v>1013</v>
       </c>
       <c r="D48" s="6">
         <v>0</v>
@@ -1885,7 +1885,7 @@
         <v>300</v>
       </c>
       <c r="C49" s="9">
-        <v>854</v>
+        <v>1536</v>
       </c>
       <c r="D49" s="9">
         <v>0</v>
@@ -1902,7 +1902,7 @@
         <v>300</v>
       </c>
       <c r="C50" s="6">
-        <v>927</v>
+        <v>1561</v>
       </c>
       <c r="D50" s="6">
         <v>0</v>
@@ -1919,7 +1919,7 @@
         <v>300</v>
       </c>
       <c r="C51" s="9">
-        <v>768</v>
+        <v>1341</v>
       </c>
       <c r="D51" s="9">
         <v>0</v>
@@ -1936,7 +1936,7 @@
         <v>300</v>
       </c>
       <c r="C52" s="6">
-        <v>691</v>
+        <v>1655</v>
       </c>
       <c r="D52" s="6">
         <v>0</v>
@@ -1953,7 +1953,7 @@
         <v>300</v>
       </c>
       <c r="C53" s="9">
-        <v>776</v>
+        <v>1508</v>
       </c>
       <c r="D53" s="9">
         <v>0</v>
@@ -1970,7 +1970,7 @@
         <v>300</v>
       </c>
       <c r="C54" s="6">
-        <v>756</v>
+        <v>1450</v>
       </c>
       <c r="D54" s="6">
         <v>0</v>
@@ -1987,7 +1987,7 @@
         <v>300</v>
       </c>
       <c r="C55" s="9">
-        <v>522</v>
+        <v>1582</v>
       </c>
       <c r="D55" s="9">
         <v>0</v>
@@ -2004,7 +2004,7 @@
         <v>300</v>
       </c>
       <c r="C56" s="6">
-        <v>887</v>
+        <v>1356</v>
       </c>
       <c r="D56" s="6">
         <v>0</v>
@@ -2021,7 +2021,7 @@
         <v>300</v>
       </c>
       <c r="C57" s="9">
-        <v>876</v>
+        <v>1675</v>
       </c>
       <c r="D57" s="9">
         <v>0</v>
@@ -2038,7 +2038,7 @@
         <v>300</v>
       </c>
       <c r="C58" s="6">
-        <v>879</v>
+        <v>1438</v>
       </c>
       <c r="D58" s="6">
         <v>0</v>
@@ -2055,7 +2055,7 @@
         <v>300</v>
       </c>
       <c r="C59" s="9">
-        <v>876</v>
+        <v>1045</v>
       </c>
       <c r="D59" s="9">
         <v>0</v>
@@ -2072,7 +2072,7 @@
         <v>300</v>
       </c>
       <c r="C60" s="6">
-        <v>852</v>
+        <v>1488</v>
       </c>
       <c r="D60" s="6">
         <v>0</v>
@@ -2089,7 +2089,7 @@
         <v>300</v>
       </c>
       <c r="C61" s="9">
-        <v>772</v>
+        <v>1435</v>
       </c>
       <c r="D61" s="9">
         <v>0</v>
@@ -2106,7 +2106,7 @@
         <v>300</v>
       </c>
       <c r="C62" s="6">
-        <v>883</v>
+        <v>1083</v>
       </c>
       <c r="D62" s="6">
         <v>0</v>
@@ -2123,12 +2123,29 @@
         <v>300</v>
       </c>
       <c r="C63" s="9">
-        <v>0</v>
+        <v>1490</v>
       </c>
       <c r="D63" s="9">
         <v>0</v>
       </c>
       <c r="E63" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="6">
+        <v>61</v>
+      </c>
+      <c r="B64" s="6">
+        <v>300</v>
+      </c>
+      <c r="C64" s="6">
+        <v>0</v>
+      </c>
+      <c r="D64" s="6">
+        <v>0</v>
+      </c>
+      <c r="E64" s="12" t="s">
         <v>71</v>
       </c>
     </row>

</xml_diff>

<commit_message>
test: run load-tests and update report
</commit_message>
<xml_diff>
--- a/testing/load-tests/Load_Test_Report.xlsx
+++ b/testing/load-tests/Load_Test_Report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1036" uniqueCount="79">
   <si>
     <t>GROWMARK BACKEND — LOAD TEST REPORT</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Start Time</t>
   </si>
   <si>
-    <t>8/7/2026, 2:41:01 PM</t>
+    <t>8/7/2026, 8:52:04 PM</t>
   </si>
   <si>
     <t>When the test started</t>
@@ -66,7 +66,7 @@
     <t>End Time</t>
   </si>
   <si>
-    <t>8/7/2026, 2:42:02 PM</t>
+    <t>8/7/2026, 8:53:05 PM</t>
   </si>
   <si>
     <t>When the test finished</t>
@@ -84,7 +84,7 @@
     <t>Average RPS</t>
   </si>
   <si>
-    <t>1205.62</t>
+    <t>1448.87</t>
   </si>
   <si>
     <t>Average requests served per second</t>
@@ -108,7 +108,7 @@
     <t>Average Response Time</t>
   </si>
   <si>
-    <t>248.58 ms</t>
+    <t>210.21 ms</t>
   </si>
   <si>
     <t>Mean time server took to respond</t>
@@ -117,7 +117,7 @@
     <t>Min Response Time</t>
   </si>
   <si>
-    <t>58 ms</t>
+    <t>59 ms</t>
   </si>
   <si>
     <t>Fastest response observed</t>
@@ -126,7 +126,7 @@
     <t>Max Response Time</t>
   </si>
   <si>
-    <t>9902 ms</t>
+    <t>9945 ms</t>
   </si>
   <si>
     <t>Slowest response observed</t>
@@ -135,7 +135,7 @@
     <t>p50 (Median)</t>
   </si>
   <si>
-    <t>127 ms</t>
+    <t>103 ms</t>
   </si>
   <si>
     <t>50% of requests responded within this time</t>
@@ -144,7 +144,7 @@
     <t>p75</t>
   </si>
   <si>
-    <t>253 ms</t>
+    <t>172 ms</t>
   </si>
   <si>
     <t>75% of requests responded within this time</t>
@@ -153,7 +153,7 @@
     <t>p99</t>
   </si>
   <si>
-    <t>1591 ms</t>
+    <t>1336 ms</t>
   </si>
   <si>
     <t>99% of requests responded within this time</t>
@@ -195,7 +195,7 @@
     <t>Total Bytes Read</t>
   </si>
   <si>
-    <t>74578.80 KB</t>
+    <t>88132.24 KB</t>
   </si>
   <si>
     <t>Total data received from the server</t>
@@ -204,7 +204,7 @@
     <t>Average Throughput</t>
   </si>
   <si>
-    <t>1243.02 KB/s</t>
+    <t>1493.82 KB/s</t>
   </si>
   <si>
     <t>Average data received per second</t>
@@ -246,10 +246,10 @@
     <t>Active — Some Errors</t>
   </si>
   <si>
-    <t>241.1</t>
-  </si>
-  <si>
-    <t>248.58</t>
+    <t>284.9</t>
+  </si>
+  <si>
+    <t>210.21</t>
   </si>
 </sst>
 </file>
@@ -867,7 +867,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="6">
-        <v>72337</v>
+        <v>85483</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>21</v>
@@ -889,7 +889,7 @@
         <v>25</v>
       </c>
       <c r="B13" s="6">
-        <v>1675</v>
+        <v>1711</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>26</v>
@@ -900,7 +900,7 @@
         <v>27</v>
       </c>
       <c r="B14" s="9">
-        <v>84</v>
+        <v>356</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>28</v>
@@ -1002,7 +1002,7 @@
         <v>52</v>
       </c>
       <c r="B24" s="6">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>53</v>
@@ -1013,7 +1013,7 @@
         <v>54</v>
       </c>
       <c r="B25" s="9">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="C25" s="10" t="s">
         <v>55</v>
@@ -1024,7 +1024,7 @@
         <v>56</v>
       </c>
       <c r="B26" s="6">
-        <v>72337</v>
+        <v>85483</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>57</v>
@@ -1075,7 +1075,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1137,7 +1137,7 @@
         <v>300</v>
       </c>
       <c r="C5" s="9">
-        <v>84</v>
+        <v>356</v>
       </c>
       <c r="D5" s="9">
         <v>0</v>
@@ -1154,7 +1154,7 @@
         <v>300</v>
       </c>
       <c r="C6" s="6">
-        <v>1199</v>
+        <v>1622</v>
       </c>
       <c r="D6" s="6">
         <v>0</v>
@@ -1171,7 +1171,7 @@
         <v>300</v>
       </c>
       <c r="C7" s="9">
-        <v>1072</v>
+        <v>1711</v>
       </c>
       <c r="D7" s="9">
         <v>0</v>
@@ -1188,7 +1188,7 @@
         <v>300</v>
       </c>
       <c r="C8" s="6">
-        <v>1226</v>
+        <v>1595</v>
       </c>
       <c r="D8" s="6">
         <v>0</v>
@@ -1205,7 +1205,7 @@
         <v>300</v>
       </c>
       <c r="C9" s="9">
-        <v>1235</v>
+        <v>1576</v>
       </c>
       <c r="D9" s="9">
         <v>0</v>
@@ -1222,7 +1222,7 @@
         <v>300</v>
       </c>
       <c r="C10" s="6">
-        <v>935</v>
+        <v>1457</v>
       </c>
       <c r="D10" s="6">
         <v>0</v>
@@ -1239,7 +1239,7 @@
         <v>300</v>
       </c>
       <c r="C11" s="9">
-        <v>1179</v>
+        <v>1552</v>
       </c>
       <c r="D11" s="9">
         <v>0</v>
@@ -1256,7 +1256,7 @@
         <v>300</v>
       </c>
       <c r="C12" s="6">
-        <v>1162</v>
+        <v>1486</v>
       </c>
       <c r="D12" s="6">
         <v>0</v>
@@ -1273,7 +1273,7 @@
         <v>300</v>
       </c>
       <c r="C13" s="9">
-        <v>1081</v>
+        <v>1517</v>
       </c>
       <c r="D13" s="9">
         <v>0</v>
@@ -1290,7 +1290,7 @@
         <v>300</v>
       </c>
       <c r="C14" s="6">
-        <v>340</v>
+        <v>1542</v>
       </c>
       <c r="D14" s="6">
         <v>0</v>
@@ -1307,7 +1307,7 @@
         <v>300</v>
       </c>
       <c r="C15" s="9">
-        <v>376</v>
+        <v>1512</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
@@ -1324,7 +1324,7 @@
         <v>300</v>
       </c>
       <c r="C16" s="6">
-        <v>827</v>
+        <v>1475</v>
       </c>
       <c r="D16" s="6">
         <v>0</v>
@@ -1341,7 +1341,7 @@
         <v>300</v>
       </c>
       <c r="C17" s="9">
-        <v>850</v>
+        <v>1541</v>
       </c>
       <c r="D17" s="9">
         <v>0</v>
@@ -1358,7 +1358,7 @@
         <v>300</v>
       </c>
       <c r="C18" s="6">
-        <v>755</v>
+        <v>1342</v>
       </c>
       <c r="D18" s="6">
         <v>0</v>
@@ -1375,7 +1375,7 @@
         <v>300</v>
       </c>
       <c r="C19" s="9">
-        <v>840</v>
+        <v>1437</v>
       </c>
       <c r="D19" s="9">
         <v>0</v>
@@ -1392,7 +1392,7 @@
         <v>300</v>
       </c>
       <c r="C20" s="6">
-        <v>939</v>
+        <v>1090</v>
       </c>
       <c r="D20" s="6">
         <v>0</v>
@@ -1409,7 +1409,7 @@
         <v>300</v>
       </c>
       <c r="C21" s="9">
-        <v>713</v>
+        <v>1687</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
@@ -1426,7 +1426,7 @@
         <v>300</v>
       </c>
       <c r="C22" s="6">
-        <v>966</v>
+        <v>1421</v>
       </c>
       <c r="D22" s="6">
         <v>0</v>
@@ -1443,7 +1443,7 @@
         <v>300</v>
       </c>
       <c r="C23" s="9">
-        <v>1138</v>
+        <v>1524</v>
       </c>
       <c r="D23" s="9">
         <v>0</v>
@@ -1460,7 +1460,7 @@
         <v>300</v>
       </c>
       <c r="C24" s="6">
-        <v>1128</v>
+        <v>1303</v>
       </c>
       <c r="D24" s="6">
         <v>0</v>
@@ -1477,7 +1477,7 @@
         <v>300</v>
       </c>
       <c r="C25" s="9">
-        <v>1247</v>
+        <v>1300</v>
       </c>
       <c r="D25" s="9">
         <v>0</v>
@@ -1494,7 +1494,7 @@
         <v>300</v>
       </c>
       <c r="C26" s="6">
-        <v>1149</v>
+        <v>1165</v>
       </c>
       <c r="D26" s="6">
         <v>0</v>
@@ -1511,7 +1511,7 @@
         <v>300</v>
       </c>
       <c r="C27" s="9">
-        <v>1402</v>
+        <v>1552</v>
       </c>
       <c r="D27" s="9">
         <v>0</v>
@@ -1528,7 +1528,7 @@
         <v>300</v>
       </c>
       <c r="C28" s="6">
-        <v>1367</v>
+        <v>1557</v>
       </c>
       <c r="D28" s="6">
         <v>0</v>
@@ -1545,7 +1545,7 @@
         <v>300</v>
       </c>
       <c r="C29" s="9">
-        <v>1538</v>
+        <v>1505</v>
       </c>
       <c r="D29" s="9">
         <v>0</v>
@@ -1562,7 +1562,7 @@
         <v>300</v>
       </c>
       <c r="C30" s="6">
-        <v>1405</v>
+        <v>811</v>
       </c>
       <c r="D30" s="6">
         <v>0</v>
@@ -1579,7 +1579,7 @@
         <v>300</v>
       </c>
       <c r="C31" s="9">
-        <v>1494</v>
+        <v>1347</v>
       </c>
       <c r="D31" s="9">
         <v>0</v>
@@ -1596,7 +1596,7 @@
         <v>300</v>
       </c>
       <c r="C32" s="6">
-        <v>1558</v>
+        <v>1382</v>
       </c>
       <c r="D32" s="6">
         <v>0</v>
@@ -1613,7 +1613,7 @@
         <v>300</v>
       </c>
       <c r="C33" s="9">
-        <v>1370</v>
+        <v>1333</v>
       </c>
       <c r="D33" s="9">
         <v>0</v>
@@ -1630,7 +1630,7 @@
         <v>300</v>
       </c>
       <c r="C34" s="6">
-        <v>815</v>
+        <v>1541</v>
       </c>
       <c r="D34" s="6">
         <v>0</v>
@@ -1647,7 +1647,7 @@
         <v>300</v>
       </c>
       <c r="C35" s="9">
-        <v>1043</v>
+        <v>1483</v>
       </c>
       <c r="D35" s="9">
         <v>0</v>
@@ -1664,7 +1664,7 @@
         <v>300</v>
       </c>
       <c r="C36" s="6">
-        <v>1287</v>
+        <v>1304</v>
       </c>
       <c r="D36" s="6">
         <v>0</v>
@@ -1681,7 +1681,7 @@
         <v>300</v>
       </c>
       <c r="C37" s="9">
-        <v>1322</v>
+        <v>1599</v>
       </c>
       <c r="D37" s="9">
         <v>0</v>
@@ -1698,7 +1698,7 @@
         <v>300</v>
       </c>
       <c r="C38" s="6">
-        <v>1451</v>
+        <v>1477</v>
       </c>
       <c r="D38" s="6">
         <v>0</v>
@@ -1715,7 +1715,7 @@
         <v>300</v>
       </c>
       <c r="C39" s="9">
-        <v>1513</v>
+        <v>1413</v>
       </c>
       <c r="D39" s="9">
         <v>0</v>
@@ -1732,7 +1732,7 @@
         <v>300</v>
       </c>
       <c r="C40" s="6">
-        <v>1443</v>
+        <v>1434</v>
       </c>
       <c r="D40" s="6">
         <v>0</v>
@@ -1749,7 +1749,7 @@
         <v>300</v>
       </c>
       <c r="C41" s="9">
-        <v>1215</v>
+        <v>1593</v>
       </c>
       <c r="D41" s="9">
         <v>0</v>
@@ -1766,7 +1766,7 @@
         <v>300</v>
       </c>
       <c r="C42" s="6">
-        <v>1466</v>
+        <v>1584</v>
       </c>
       <c r="D42" s="6">
         <v>0</v>
@@ -1783,7 +1783,7 @@
         <v>300</v>
       </c>
       <c r="C43" s="9">
-        <v>1472</v>
+        <v>1552</v>
       </c>
       <c r="D43" s="9">
         <v>0</v>
@@ -1800,7 +1800,7 @@
         <v>300</v>
       </c>
       <c r="C44" s="6">
-        <v>1582</v>
+        <v>1459</v>
       </c>
       <c r="D44" s="6">
         <v>0</v>
@@ -1817,7 +1817,7 @@
         <v>300</v>
       </c>
       <c r="C45" s="9">
-        <v>1565</v>
+        <v>1586</v>
       </c>
       <c r="D45" s="9">
         <v>0</v>
@@ -1834,7 +1834,7 @@
         <v>300</v>
       </c>
       <c r="C46" s="6">
-        <v>1326</v>
+        <v>1553</v>
       </c>
       <c r="D46" s="6">
         <v>0</v>
@@ -1851,7 +1851,7 @@
         <v>300</v>
       </c>
       <c r="C47" s="9">
-        <v>1606</v>
+        <v>1552</v>
       </c>
       <c r="D47" s="9">
         <v>0</v>
@@ -1868,7 +1868,7 @@
         <v>300</v>
       </c>
       <c r="C48" s="6">
-        <v>1013</v>
+        <v>1543</v>
       </c>
       <c r="D48" s="6">
         <v>0</v>
@@ -1885,7 +1885,7 @@
         <v>300</v>
       </c>
       <c r="C49" s="9">
-        <v>1536</v>
+        <v>1670</v>
       </c>
       <c r="D49" s="9">
         <v>0</v>
@@ -1902,7 +1902,7 @@
         <v>300</v>
       </c>
       <c r="C50" s="6">
-        <v>1561</v>
+        <v>1567</v>
       </c>
       <c r="D50" s="6">
         <v>0</v>
@@ -1919,7 +1919,7 @@
         <v>300</v>
       </c>
       <c r="C51" s="9">
-        <v>1341</v>
+        <v>1575</v>
       </c>
       <c r="D51" s="9">
         <v>0</v>
@@ -1936,7 +1936,7 @@
         <v>300</v>
       </c>
       <c r="C52" s="6">
-        <v>1655</v>
+        <v>1657</v>
       </c>
       <c r="D52" s="6">
         <v>0</v>
@@ -1953,7 +1953,7 @@
         <v>300</v>
       </c>
       <c r="C53" s="9">
-        <v>1508</v>
+        <v>1571</v>
       </c>
       <c r="D53" s="9">
         <v>0</v>
@@ -1970,7 +1970,7 @@
         <v>300</v>
       </c>
       <c r="C54" s="6">
-        <v>1450</v>
+        <v>1603</v>
       </c>
       <c r="D54" s="6">
         <v>0</v>
@@ -1987,7 +1987,7 @@
         <v>300</v>
       </c>
       <c r="C55" s="9">
-        <v>1582</v>
+        <v>1592</v>
       </c>
       <c r="D55" s="9">
         <v>0</v>
@@ -2004,7 +2004,7 @@
         <v>300</v>
       </c>
       <c r="C56" s="6">
-        <v>1356</v>
+        <v>1570</v>
       </c>
       <c r="D56" s="6">
         <v>0</v>
@@ -2021,7 +2021,7 @@
         <v>300</v>
       </c>
       <c r="C57" s="9">
-        <v>1675</v>
+        <v>1522</v>
       </c>
       <c r="D57" s="9">
         <v>0</v>
@@ -2038,7 +2038,7 @@
         <v>300</v>
       </c>
       <c r="C58" s="6">
-        <v>1438</v>
+        <v>1585</v>
       </c>
       <c r="D58" s="6">
         <v>0</v>
@@ -2055,7 +2055,7 @@
         <v>300</v>
       </c>
       <c r="C59" s="9">
-        <v>1045</v>
+        <v>1590</v>
       </c>
       <c r="D59" s="9">
         <v>0</v>
@@ -2072,7 +2072,7 @@
         <v>300</v>
       </c>
       <c r="C60" s="6">
-        <v>1488</v>
+        <v>1534</v>
       </c>
       <c r="D60" s="6">
         <v>0</v>
@@ -2089,7 +2089,7 @@
         <v>300</v>
       </c>
       <c r="C61" s="9">
-        <v>1435</v>
+        <v>1567</v>
       </c>
       <c r="D61" s="9">
         <v>0</v>
@@ -2106,7 +2106,7 @@
         <v>300</v>
       </c>
       <c r="C62" s="6">
-        <v>1083</v>
+        <v>1509</v>
       </c>
       <c r="D62" s="6">
         <v>0</v>
@@ -2123,29 +2123,12 @@
         <v>300</v>
       </c>
       <c r="C63" s="9">
-        <v>1490</v>
+        <v>0</v>
       </c>
       <c r="D63" s="9">
         <v>0</v>
       </c>
       <c r="E63" s="12" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="64" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="6">
-        <v>61</v>
-      </c>
-      <c r="B64" s="6">
-        <v>300</v>
-      </c>
-      <c r="C64" s="6">
-        <v>0</v>
-      </c>
-      <c r="D64" s="6">
-        <v>0</v>
-      </c>
-      <c r="E64" s="12" t="s">
         <v>71</v>
       </c>
     </row>

</xml_diff>